<commit_message>
Template guide says 10 seconds; no hair outside the space helmet
- 7주차_영단어.xlsx (and its [템플릿 받기] copy): the 안내 sheet now says a blank 시간(초) is 10 seconds and a blank
  세트 names the event after the file. Only those two lines changed.
- The space helmet is sealed glass, so long, braided and ponytail hair no longer pokes out of it (review finding).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/week7.xlsx
+++ b/public/templates/week7.xlsx
@@ -35,7 +35,7 @@
     <x:t>학생 명단은 이 파일에 넣지 않아요. 선생님 화면 [학생·기기]에서 반을 만들면, 학생이 처음 접속할 때 반·번호·이름을 직접 써서 등록해요.</x:t>
   </x:si>
   <x:si>
-    <x:t>세트 (선택): 비워 두면 올린 날짜로 이벤트가 생겨요. (예: 10-29 퀴즈)</x:t>
+    <x:t>세트 (선택): 비워 두면 파일 이름으로 이벤트가 생겨요. (예: 7주차_영단어.xlsx → 7주차_영단어) 한 파일을 여러 퀴즈로 나눌 때만 쓰세요.</x:t>
   </x:si>
   <x:si>
     <x:t>상태 (선택): 사용(기본) · 검토(저장만 하고 출제 안 함) · 보관(숨김)</x:t>
@@ -68,7 +68,7 @@
     <x:t>객관식 정답은 번호(1~4), OX는 O 또는 X, 단답형은 답 (여러 답은 a|b).</x:t>
   </x:si>
   <x:si>
-    <x:t>시간(초) (선택): 비워 두면 15초입니다. 특별히 오래 걸리는 단어만 숫자를 쓰세요.</x:t>
+    <x:t>시간(초) (선택): 비워 두면 10초예요. 오래 걸리는 단어만 숫자를 쓰세요.</x:t>
   </x:si>
   <x:si>
     <x:t>'단어장' 시트에 단어와 뜻 두 칸만 채우세요. 객관식 문제와 오답 보기는 앱이 만들어요.</x:t>

</xml_diff>